<commit_message>
UAT pack: add case E-09 — payment-confirmation upload on disbursement (83 cases)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Proximate_UAT_Test_Pack_July2026.xlsx
+++ b/docs/Proximate_UAT_Test_Pack_July2026.xlsx
@@ -4272,7 +4272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4682,9 +4682,53 @@
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>E-09</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>ob@proximate.org</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>E-02 done ({D1} disbursed)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>1. Open disbursement {D1}.
+2. Find the 'Payment confirmations' card.
+3. Upload UAT_Evidence_Photo_3.jpg as the hawala/payment-app receipt (kind: Payment confirmation).
+4. Refresh the page and download the file back.</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>UAT_Evidence_Photo_3.jpg (stands in for the government payment-app screenshot)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>This mirrors the real workflow: confirm with the hawala, then save the government payment-app confirmation against the SPECIFIC transfer. The file uploads, is listed on the disbursement with a 'Payment confirmation' badge, survives a refresh, and downloads intact. The upload is recorded in the audit chain.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr"/>
+      <c r="K10" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
UAT pack: add B-03 round activation dual sign-off case (84 cases)
Opening a round is multi-sig (2 OB signatures + COI declaration);
the pack now exercises it explicitly and unblocks the downstream
cases that need an active round.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Proximate_UAT_Test_Pack_July2026.xlsx
+++ b/docs/Proximate_UAT_Test_Pack_July2026.xlsx
@@ -2894,7 +2894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3064,12 +3064,12 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>OB + OB #2</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>ob@proximate.org</t>
+          <t>ob@proximate.org, then ob2@proximate.org</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -3079,18 +3079,20 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>1. On round {R}, click through all tabs.
-2. Check the journey strip at the top.</t>
+          <t>1. On round {R}, submit it for signature (draft → in review).
+2. As ob@proximate.org, click Sign: tick the no-conflict-of-interest declaration and add note 'UAT sign-off 1'.
+3. In a second window, log in as ob2@proximate.org, open round {R} and Sign with note 'UAT sign-off 2'.
+4. Watch the round status after the second signature.</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Round {R}</t>
+          <t>Notes prefixed 'UAT'</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Five tabs render without errors. The journey strip highlights the current stage and shows what comes next in plain language.</t>
+          <t>Opening a round is a governed decision: it takes TWO Oversight Body sign-offs, each recording the signer's name, time, no-COI declaration and note. One signer alone cannot activate; not ticking the COI box records a recusal instead of an approval. After the second signature the round becomes Active automatically. The signature roster shows both decisions and both appear in the audit chain (case H-04).</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr"/>
@@ -3116,24 +3118,23 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>B-03 done</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/crisis-selector/.
-2. Add a manual crisis signal: severity High, note 'UAT signal — Blue Nile access constraint (test entry)'.
-3. Save and review the list.</t>
+          <t>1. On round {R}, click through all tabs.
+2. Check the journey strip at the top.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Signal note as in steps</t>
+          <t>Round {R}</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Signal saves and appears in the list with a severity band (colour-coded). The page explains its purpose (feeding round triggers) in a header. Do NOT start a round from here.</t>
+          <t>Five tabs render without errors. The journey strip highlights the current stage and shows what comes next in plain language.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr"/>
@@ -3159,23 +3160,24 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>B-02 done</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>1. In the rounds register, click a status filter chip (e.g. Active/Draft).
-2. Copy the page URL, open it in a new tab.</t>
+          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/crisis-selector/.
+2. Add a manual crisis signal: severity High, note 'UAT signal — Blue Nile access constraint (test entry)'.
+3. Save and review the list.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Signal note as in steps</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>The list filters; the URL contains the filter and reproduces the same filtered view in the new tab (shareable link).</t>
+          <t>Signal saves and appears in the list with a severity band (colour-coded). The page explains its purpose (feeding round triggers) in a header. Do NOT start a round from here.</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
@@ -3191,12 +3193,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Donor</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>uat.donor@proximate.org</t>
+          <t>ob@proximate.org</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -3206,8 +3208,8 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1. Log in as the donor (fresh window).
-2. Open the donor dashboard.</t>
+          <t>1. In the rounds register, click a status filter chip (e.g. Active/Draft).
+2. Copy the page URL, open it in a new tab.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -3217,7 +3219,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>The new round 'UAT Round — July 2026 (Team)' is now visible to the donor automatically — because UAT Donor Foundation funds it. Round 8 is still there. Nothing else (no Blue Nile).</t>
+          <t>The list filters; the URL contains the filter and reproduces the same filtered view in the new tab (shareable link).</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
@@ -3233,12 +3235,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>Donor</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>ob@proximate.org</t>
+          <t>uat.donor@proximate.org</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -3248,19 +3250,18 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1. On round {R}, find the panel selection / community panel section.
-2. Add candidate 'Halima Adam Koko' and upload UAT_Panelist_CV_Halima.pdf as her CV.
-3. Generate/copy the public voting link.</t>
+          <t>1. Log in as the donor (fresh window).
+2. Open the donor dashboard.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>UAT_Panelist_CV_Halima.pdf</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Candidate saves with CV attached. A public voting link (token URL) is produced for community panel selection.</t>
+          <t>The new round 'UAT Round — July 2026 (Team)' is now visible to the donor automatically — because UAT Donor Foundation funds it. Round 8 is still there. Nothing else (no Blue Nile).</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr"/>
@@ -3276,34 +3277,34 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Public voter</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>— incognito —</t>
+          <t>ob@proximate.org</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>B-07 done</t>
+          <t>B-03 done</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>1. Open the voting link from B-07 in an incognito window.
-2. Cast a vote for Halima.
-3. Try to vote a second time from the same link.</t>
+          <t>1. On round {R}, find the panel selection / community panel section.
+2. Add candidate 'Halima Adam Koko' and upload UAT_Panelist_CV_Halima.pdf as her CV.
+3. Generate/copy the public voting link.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Voting token link</t>
+          <t>UAT_Panelist_CV_Halima.pdf</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Vote page loads without login (Arabic/English available), vote is accepted and confirmed. A second vote from the same token is prevented or clearly handled per design — no double count.</t>
+          <t>Candidate saves with CV attached. A public voting link (token URL) is produced for community panel selection.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
@@ -3311,9 +3312,52 @@
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Public voter</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>— incognito —</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>B-08 done</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>1. Open the voting link from B-08 in an incognito window.
+2. Cast a vote for Halima.
+3. Try to vote a second time from the same link.</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Voting token link</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Vote page loads without login (Arabic/English available), vote is accepted and confirmed. A second vote from the same token is prevented or clearly handled per design — no double count.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr"/>
+      <c r="K10" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3505,7 +3549,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>C-02, B-02 done</t>
+          <t>C-02, B-03 done (round {R} active)</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">

</xml_diff>

<commit_message>
UAT pack: primary URL is now https://proximate.kuja.org (custom domain live)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Proximate_UAT_Test_Pack_July2026.xlsx
+++ b/docs/Proximate_UAT_Test_Pack_July2026.xlsx
@@ -542,21 +542,21 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>URL: https://web-production-6f8a.up.railway.app</t>
+          <t>URL: https://proximate.kuja.org</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>ALWAYS log in via this exact link: https://web-production-6f8a.up.railway.app/login/?network=proximate</t>
+          <t>Log in at: https://proximate.kuja.org/login/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>(The plain /login page clears the Proximate context — if you ever see marketplace branding, re-open the link above.) If proximate.kuja.org has gone live on your network, you can use it instead and drop the ?network=proximate part.</t>
+          <t>This domain always shows the Proximate console — no special links needed. Backup URL if the domain is ever unreachable: https://web-production-6f8a.up.railway.app/login/?network=proximate (on the backup URL, always use that exact link).</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate-grievance/ in incognito.
+          <t>1. Open https://proximate.kuja.org/proximate-grievance/ in incognito.
 2. Submit a grievance: 'UAT grievance — test entry, please triage as test'. Leave contact optional/empty.
 3. Note the reference code.</t>
         </is>
@@ -885,7 +885,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/admin/audit-chain/.
+          <t>1. Open https://proximate.kuja.org/admin/audit-chain/.
 2. Filter/scan for today's UAT actions (round created, disbursement signed, package published…).
 3. Expand two rows.</t>
         </is>
@@ -970,7 +970,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/ in incognito (public transparency page).</t>
+          <t>1. Open https://proximate.kuja.org/proximate/ in incognito (public transparency page).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/settings/notifications/.
+          <t>1. Open https://proximate.kuja.org/settings/notifications/.
 2. Review the category groups.
 3. Toggle one category off, save, refresh, toggle it back on.</t>
         </is>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/settings/.
+          <t>1. Open https://proximate.kuja.org/settings/.
 2. Review the hub: profile, language, theme, low-bandwidth, links to notifications/security.
 3. Click Settings from the sidebar too.</t>
         </is>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/login/?network=proximate
+          <t>1. Open https://proximate.kuja.org/login/
 2. Log in.
 3. Look at the left sidebar and the top of the page.</t>
         </is>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/login/?network=proximate in a fresh browser/profile.
+          <t>1. Open https://proximate.kuja.org/login/ in a fresh browser/profile.
 2. Log in as the donor.
 3. Review what is visible.</t>
         </is>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/login/?network=proximate in a fresh browser/profile.
+          <t>1. Open https://proximate.kuja.org/login/ in a fresh browser/profile.
 2. Log in.
 3. Review what is visible.</t>
         </is>
@@ -2563,8 +2563,8 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>1. Paste https://web-production-6f8a.up.railway.app/proximate/admin/ into the address bar.
-2. Then try https://web-production-6f8a.up.railway.app/proximate/admin/partners/.</t>
+          <t>1. Paste https://proximate.kuja.org/proximate/admin/ into the address bar.
+2. Then try https://proximate.kuja.org/proximate/admin/partners/.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -2605,8 +2605,8 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1. Paste https://web-production-6f8a.up.railway.app/proximate/disbursements/ into the address bar.
-2. Then try https://web-production-6f8a.up.railway.app/proximate/rounds/.</t>
+          <t>1. Paste https://proximate.kuja.org/proximate/disbursements/ into the address bar.
+2. Then try https://proximate.kuja.org/proximate/rounds/.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/admin/ while logged out.</t>
+          <t>1. Open https://proximate.kuja.org/proximate/admin/ while logged out.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -2815,8 +2815,8 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>1. Log in via https://web-production-6f8a.up.railway.app/login/?network=proximate.
-2. Open https://web-production-6f8a.up.railway.app/admin/audit-chain/.
+          <t>1. Log in via https://proximate.kuja.org/login/.
+2. Open https://proximate.kuja.org/admin/audit-chain/.
 3. Expand any recent row.</t>
         </is>
       </c>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/login/?network=proximate.
+          <t>1. Open https://proximate.kuja.org/login/.
 2. Enter ob@proximate.org with password 'wrongpass' and submit.
 3. Then log in with the correct password.</t>
         </is>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/grants/.
+          <t>1. Open https://proximate.kuja.org/proximate/grants/.
 2. Choose to add/upload a grant and select UAT_Grant_Agreement_UATDonor.pdf.
 3. Wait for the AI extraction wizard.
 4. Review the extracted fields, correct anything wrong, confirm/save.</t>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/rounds/.
+          <t>1. Open https://proximate.kuja.org/proximate/rounds/.
 2. Click New round.
 3. Trigger: donor commitment. Donor: select 'UAT Donor Foundation' from the dropdown.
 4. Title: 'UAT Round — July 2026 (Team)'. Envelope: USD 20,000.
@@ -3165,7 +3165,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/crisis-selector/.
+          <t>1. Open https://proximate.kuja.org/proximate/crisis-selector/.
 2. Add a manual crisis signal: severity High, note 'UAT signal — Blue Nile access constraint (test entry)'.
 3. Save and review the list.</t>
         </is>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate-nominate/ in incognito.
+          <t>1. Open https://proximate.kuja.org/proximate-nominate/ in incognito.
 2. Fill the self-nomination for 'Amal Relief Initiative (UAT)': location Ed Damazin, phone +249 91 000 0042, email uat.partner.amal@example.org, brief description 'UAT test nomination — community relief group'.
 3. Submit.</t>
         </is>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/admin/partners/.
+          <t>1. Open https://proximate.kuja.org/proximate/admin/partners/.
 2. Search 'Amal'.
 3. Open the partner page and note its ID into 'Runtime values' as {P}.
 4. Check the Due diligence tab.</t>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate-endorse/ in incognito (public endorser sign-up).
+          <t>1. Open https://proximate.kuja.org/proximate-endorse/ in incognito (public endorser sign-up).
 2. Register 'UAT Endorser Omar', phone +249 91 000 0077, community Ed Damazin, set a password.
 3. Submit.</t>
         </is>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/disbursements/.
+          <t>1. Open https://proximate.kuja.org/proximate/disbursements/.
 2. Use the status filter chips and search.
 3. Scroll/paginate if more than one page.</t>
         </is>
@@ -4707,7 +4707,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>1. Open https://web-production-6f8a.up.railway.app/proximate/disbursements/24/.
+          <t>1. Open https://proximate.kuja.org/proximate/disbursements/24/.
 2. LOOK ONLY — do not click any action.</t>
         </is>
       </c>
@@ -5566,7 +5566,7 @@
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>1. Log in as the donor (fresh window).
-2. Open https://web-production-6f8a.up.railway.app/proximate/reports/ and open the new package for round {R}.</t>
+2. Open https://proximate.kuja.org/proximate/reports/ and open the new package for round {R}.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>1. Try opening a package that belongs to a round this donor does not fund — paste https://web-production-6f8a.up.railway.app/proximate/reports/1/ (and /2/) into the address bar.</t>
+          <t>1. Try opening a package that belongs to a round this donor does not fund — paste https://proximate.kuja.org/proximate/reports/1/ (and /2/) into the address bar.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">

</xml_diff>